<commit_message>
Ruta A v4 «Montecristo × Hoyo de Monterrey»: art vectorial sense errors de text
Anelles Nº 1–3, segona anella «Pliego de autor», emblema, vista i marca a foc
en vectorial (_build/brand_v4.py, text en traçats). Maqueta de la caixa amb la
marca gravada per homografia. Dossier, brief d'identitat, pla de negoci, Prompt
Pack i README actualitzats; fonts S59–S61. Cua de fotos sense text per al 14/10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Cf1VjW9mqckGqcvuVgoNK
</commit_message>
<xml_diff>
--- a/PROYECTO_CIGARS_CUBA_2027/09_RESEARCH/Source Register.xlsx
+++ b/PROYECTO_CIGARS_CUBA_2027/09_RESEARCH/Source Register.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="311">
   <si>
     <t xml:space="preserve">Registro de fuentes — consulta 10/10/2026</t>
   </si>
@@ -812,6 +812,42 @@
   </si>
   <si>
     <t xml:space="preserve">Bolívar (creada en 1902): la imagen de su epónimo, Simón Bolívar, forma parte de la marca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cigar Aficionado — How to spot a fake Hoyo de Monterrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.cigaraficionado.com/article/how-to-spot-a-fake-hoyo-de-monterrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anilla estándar de Hoyo de Monterrey: mayoritariamente blanca, con un logotipo rojo central y el nombre en letras blancas; la línea Epicure añade una segunda anilla.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simply Cigars — Montecristo 80th anniversary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.simplycigars.co.uk/guide/montecristo-80th-anniversary-cubas-best-selling-brand-1907/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anilla de Montecristo: campo marrón con filigrana de oro y bordes blancos; la flor de lis central va en relieve de oro desde 2013.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JJ Fox — 1935, the year of Montecristo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://jjfox.co.uk/blog/cigar-brands/1935-the-year-of-montecristo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montecristo nace en 1935 (Alonso Menéndez, fábrica Particulares); su emblema es un triángulo de espadas en torno a una flor de lis.</t>
   </si>
   <si>
     <t xml:space="preserve">S54</t>
@@ -1317,7 +1353,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2672,7 +2708,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
         <v>264</v>
       </c>
@@ -2683,10 +2719,10 @@
         <v>266</v>
       </c>
       <c r="D62" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" s="4" t="s">
         <v>267</v>
-      </c>
-      <c r="E62" s="4" t="s">
-        <v>268</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>20</v>
@@ -2697,19 +2733,19 @@
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="B63" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="B63" s="4" t="s">
+      <c r="C63" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="C63" s="4" t="s">
+      <c r="D63" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" s="4" t="s">
         <v>271</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E63" s="4" t="s">
-        <v>273</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>20</v>
@@ -2720,42 +2756,42 @@
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="C64" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="D64" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E64" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="C64" s="4" t="s">
+      <c r="F64" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="D64" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E64" s="4" t="s">
+      <c r="B65" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="F64" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G64" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="4" t="s">
+      <c r="C65" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="D65" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="C65" s="4" t="s">
+      <c r="E65" s="4" t="s">
         <v>280</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E65" s="4" t="s">
-        <v>281</v>
       </c>
       <c r="F65" s="4" t="s">
         <v>20</v>
@@ -2766,16 +2802,16 @@
     </row>
     <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B66" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="B66" s="4" t="s">
+      <c r="C66" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="C66" s="4" t="s">
+      <c r="D66" s="4" t="s">
         <v>284</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>272</v>
       </c>
       <c r="E66" s="4" t="s">
         <v>285</v>
@@ -2787,7 +2823,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
         <v>286</v>
       </c>
@@ -2798,7 +2834,7 @@
         <v>288</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="E67" s="4" t="s">
         <v>289</v>
@@ -2810,7 +2846,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
         <v>290</v>
       </c>
@@ -2821,7 +2857,7 @@
         <v>292</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="E68" s="4" t="s">
         <v>293</v>
@@ -2833,7 +2869,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
         <v>294</v>
       </c>
@@ -2844,15 +2880,84 @@
         <v>296</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="E69" s="4" t="s">
         <v>297</v>
       </c>
       <c r="F69" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="G69" s="4" t="s">
+      <c r="B70" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="F70" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G70" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G71" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="G72" s="4" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>